<commit_message>
up via la classe 25/03
</commit_message>
<xml_diff>
--- a/Vari.xlsx
+++ b/Vari.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\okmen\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\okmen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086C958A-BF39-466A-B817-715527AD9F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253E0BA3-18EE-43BB-B6DD-23FA0E5CC53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2D01C2EE-179F-4AB8-94CB-C0F2827DB6D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2D01C2EE-179F-4AB8-94CB-C0F2827DB6D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="175">
   <si>
     <t>Nom de la route</t>
   </si>
@@ -274,9 +274,6 @@
     <t>{message}</t>
   </si>
   <si>
-    <t>Désactive le compte d'un tiers.</t>
-  </si>
-  <si>
     <t>/games</t>
   </si>
   <si>
@@ -379,9 +376,6 @@
     <t>PATCH/users/:id/role</t>
   </si>
   <si>
-    <t>DELETE/users/:id</t>
-  </si>
-  <si>
     <t>POST/teams</t>
   </si>
   <si>
@@ -389,12 +383,6 @@
   </si>
   <si>
     <t>AuthDTO</t>
-  </si>
-  <si>
-    <t>401 (Invalid creds)</t>
-  </si>
-  <si>
-    <t>400 (Input), 409 (Conflict)</t>
   </si>
   <si>
     <r>
@@ -474,21 +462,12 @@
     <t>Module 1 : Users</t>
   </si>
   <si>
-    <t>Module 2 gestion des matchs : Games</t>
-  </si>
-  <si>
     <t>No content</t>
   </si>
   <si>
     <t>Module 3 :  Teams</t>
   </si>
   <si>
-    <t>GET/teams/id</t>
-  </si>
-  <si>
-    <t>Récupère information d'une équipe</t>
-  </si>
-  <si>
     <t>/teams/id</t>
   </si>
   <si>
@@ -498,21 +477,9 @@
     <t>mise à jour les informations d'une équipe et seulement l'entraineur peut modifier</t>
   </si>
   <si>
-    <t>GET /user/id/teams</t>
-  </si>
-  <si>
-    <t>/teams/id/teams</t>
-  </si>
-  <si>
     <t>fields</t>
   </si>
   <si>
-    <t>user authenthifié (proptietaire)</t>
-  </si>
-  <si>
-    <t>récupère les informations d'un user et les donneés complementaires, les matchs etc..</t>
-  </si>
-  <si>
     <t>teams</t>
   </si>
   <si>
@@ -541,9 +508,6 @@
   </si>
   <si>
     <t>GET /games</t>
-  </si>
-  <si>
-    <t>GET /games/id</t>
   </si>
   <si>
     <t>games</t>
@@ -602,10 +566,34 @@
     <t>GET /fields</t>
   </si>
   <si>
-    <t>/games/id</t>
-  </si>
-  <si>
-    <t>GET /users (admin)</t>
+    <t>Module 2  : Games</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /users </t>
+  </si>
+  <si>
+    <t>GET/users/shorts</t>
+  </si>
+  <si>
+    <t>/users/shorts</t>
+  </si>
+  <si>
+    <t>GET  /  games</t>
+  </si>
+  <si>
+    <t>liste des info basics a propos des parties,</t>
+  </si>
+  <si>
+    <t>400 (données invalide)</t>
+  </si>
+  <si>
+    <t>400 (Input), 401 (invalide)</t>
+  </si>
+  <si>
+    <t>401(invalide)</t>
+  </si>
+  <si>
+    <t>404 (Not found); 401(invalide)</t>
   </si>
 </sst>
 </file>
@@ -1357,19 +1345,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6251F74D-515E-4B84-9C96-1B746F7F8599}">
   <sheetPr codeName="Feuil1"/>
   <dimension ref="A5:K30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.375" customWidth="1"/>
-    <col min="2" max="2" width="13.625" customWidth="1"/>
-    <col min="3" max="3" width="17.875" customWidth="1"/>
-    <col min="4" max="4" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.375" customWidth="1"/>
-    <col min="6" max="6" width="33.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.375" customWidth="1"/>
-    <col min="8" max="8" width="28.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="54.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="38.625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="33.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" customWidth="1"/>
+    <col min="8" max="8" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="33.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:11" ht="18">
@@ -1787,19 +1775,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E662E712-5C8B-461C-9C80-338D1AA5A420}">
   <sheetPr codeName="Feuil2"/>
   <dimension ref="A3:K66"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="23.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.75" customWidth="1"/>
-    <col min="6" max="6" width="26.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="58.625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="33.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="58.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:11" ht="18">
@@ -1837,14 +1825,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15">
+    <row r="4" spans="1:11">
       <c r="A4" s="21" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B5" s="38" t="s">
         <v>34</v>
@@ -1868,10 +1856,10 @@
         <v>58</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>117</v>
+        <v>171</v>
       </c>
       <c r="K5" t="s">
         <v>59</v>
@@ -1897,7 +1885,7 @@
         <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="H6" t="s">
         <v>60</v>
@@ -1906,7 +1894,7 @@
         <v>61</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>118</v>
+        <v>172</v>
       </c>
       <c r="K6" t="s">
         <v>62</v>
@@ -1914,7 +1902,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>167</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -1923,7 +1911,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>31</v>
+        <v>168</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>13</v>
@@ -1941,15 +1929,15 @@
         <v>63</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>13</v>
+        <v>173</v>
       </c>
       <c r="K7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" ht="40.200000000000003">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B8" s="38" t="s">
         <v>40</v>
@@ -1964,7 +1952,7 @@
         <v>13</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G8" t="s">
         <v>41</v>
@@ -1973,10 +1961,10 @@
         <v>13</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>121</v>
+        <v>174</v>
       </c>
       <c r="K8" t="s">
         <v>66</v>
@@ -1984,7 +1972,7 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>40</v>
@@ -1996,7 +1984,7 @@
         <v>67</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>13</v>
@@ -2011,7 +1999,7 @@
         <v>61</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K9" t="s">
         <v>68</v>
@@ -2019,7 +2007,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="24" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>40</v>
@@ -2028,10 +2016,10 @@
         <v>56</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F10" s="27" t="s">
         <v>13</v>
@@ -2046,7 +2034,7 @@
         <v>61</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="K10" t="s">
         <v>71</v>
@@ -2054,7 +2042,7 @@
     </row>
     <row r="11" spans="1:11" s="38" customFormat="1">
       <c r="A11" s="38" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="B11" s="38" t="s">
         <v>40</v>
@@ -2069,15 +2057,15 @@
         <v>73</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="K11" s="38" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>40</v>
@@ -2089,7 +2077,7 @@
         <v>72</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>13</v>
@@ -2104,7 +2092,7 @@
         <v>61</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K12" s="12" t="s">
         <v>75</v>
@@ -2112,7 +2100,7 @@
     </row>
     <row r="13" spans="1:11" s="38" customFormat="1">
       <c r="A13" s="35" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="B13" s="35" t="s">
         <v>40</v>
@@ -2121,16 +2109,16 @@
         <v>69</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F13" s="36" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="H13" s="35" t="s">
         <v>13</v>
@@ -2139,50 +2127,28 @@
         <v>77</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="K13" s="40" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="H14" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="J14" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" s="24" customFormat="1" ht="15">
+      <c r="A14" s="30"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="12"/>
+    </row>
+    <row r="15" spans="1:11" s="24" customFormat="1">
       <c r="A15" s="31" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2197,19 +2163,19 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="32" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C16" s="32" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>177</v>
+        <v>78</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>122</v>
+        <v>13</v>
       </c>
       <c r="F16" s="32" t="s">
         <v>13</v>
@@ -2217,25 +2183,27 @@
       <c r="G16" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32" t="s">
+        <v>79</v>
+      </c>
       <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
+      <c r="K16" s="32" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="12" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>13</v>
@@ -2250,27 +2218,27 @@
         <v>13</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J17" s="11" t="s">
         <v>13</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="12" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B18" s="32" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>18</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="11" t="s">
@@ -2283,30 +2251,30 @@
         <v>13</v>
       </c>
       <c r="I18" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="K18" s="12" t="s">
         <v>82</v>
-      </c>
-      <c r="J18" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="K18" s="12" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="12" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>13</v>
@@ -2315,68 +2283,68 @@
         <v>41</v>
       </c>
       <c r="H19" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="K19" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="K19" s="12" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="12" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>69</v>
       </c>
       <c r="D20" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="12" t="s">
+      <c r="H20" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="I20" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="K20" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="I20" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="J20" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="K20" s="12" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="12" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>69</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>13</v>
@@ -2385,33 +2353,33 @@
         <v>41</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I21" s="11" t="s">
         <v>77</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="12" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B22" s="32" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C22" s="32" t="s">
         <v>76</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F22" s="11" t="s">
         <v>13</v>
@@ -2423,18 +2391,18 @@
         <v>13</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>13</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" s="22" customFormat="1" ht="15">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="22" customFormat="1">
       <c r="A23" s="33" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -2448,50 +2416,30 @@
       <c r="K23" s="12"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="B24" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="C24" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="32" t="s">
-        <v>143</v>
-      </c>
-      <c r="E24" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="F24" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="34" t="s">
-        <v>17</v>
-      </c>
+      <c r="A24" s="32"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
       <c r="H24" s="34"/>
-      <c r="I24" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="J24" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="K24" s="34" t="s">
-        <v>142</v>
-      </c>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34"/>
+      <c r="K24" s="34"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="6" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>13</v>
@@ -2506,63 +2454,63 @@
         <v>13</v>
       </c>
       <c r="I25" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="K25" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="16" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="I26" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="I26" s="16" t="s">
+      <c r="J26" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="K26" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="J26" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="6" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>13</v>
@@ -2574,30 +2522,30 @@
         <v>13</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J27" s="15" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:11" s="24" customFormat="1">
       <c r="A28" s="7" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>76</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F28" s="16" t="s">
         <v>13</v>
@@ -2609,82 +2557,64 @@
         <v>13</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>13</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="24" customFormat="1">
       <c r="A29" s="32" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="B29" s="32" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C29" s="32" t="s">
         <v>56</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E29" s="32" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F29" s="32" t="s">
         <v>13</v>
       </c>
       <c r="G29" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="H29" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="H29" s="32" t="s">
-        <v>99</v>
-      </c>
       <c r="I29" s="32" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="J29" s="32"/>
       <c r="K29" s="32" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="B30" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="C30" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="F30" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="32" t="s">
-        <v>149</v>
-      </c>
+      <c r="A30" s="32"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
       <c r="H30" s="32"/>
-      <c r="I30" s="32" t="s">
-        <v>96</v>
-      </c>
+      <c r="I30" s="32"/>
       <c r="J30" s="32"/>
-      <c r="K30" s="32" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="15">
+      <c r="K30" s="32"/>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" s="33" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -2699,16 +2629,16 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E32" s="14" t="s">
         <v>13</v>
@@ -2720,16 +2650,16 @@
         <v>73</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I32" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="I32" s="14" t="s">
+      <c r="J32" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="K32" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="J32" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2753,16 +2683,16 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="6" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>13</v>
@@ -2771,54 +2701,54 @@
         <v>13</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>13</v>
       </c>
       <c r="I34" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="J34" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="K34" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="J34" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="18" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="C35" s="19" t="s">
         <v>12</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H35" s="12" t="s">
         <v>13</v>
       </c>
       <c r="I35" s="39" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J35" s="12">
         <v>401</v>
       </c>
       <c r="K35" s="20" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:11">

</xml_diff>

<commit_message>
Auth up à regarder/verifier
</commit_message>
<xml_diff>
--- a/Vari.xlsx
+++ b/Vari.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\okmen\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\okmen\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253E0BA3-18EE-43BB-B6DD-23FA0E5CC53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3C901CF-C1D5-4A61-BAA9-AF2EC27330B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2D01C2EE-179F-4AB8-94CB-C0F2827DB6D3}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2D01C2EE-179F-4AB8-94CB-C0F2827DB6D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="179">
   <si>
     <t>Nom de la route</t>
   </si>
@@ -411,46 +411,10 @@
     <t>UserDTO[]</t>
   </si>
   <si>
-    <t>404 (Not found)</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
-    <t>400 (Bad input)</t>
-  </si>
-  <si>
-    <t>403 (Forbidden)</t>
-  </si>
-  <si>
-    <t>403 (Admin status)</t>
-  </si>
-  <si>
-    <t>400, 422 (Started)</t>
-  </si>
-  <si>
-    <t>400 (Invalid trans.)</t>
-  </si>
-  <si>
-    <t>403 (Not started)</t>
-  </si>
-  <si>
-    <t>400 (Bad sport)</t>
-  </si>
-  <si>
-    <t>409 (Already in)</t>
-  </si>
-  <si>
-    <t>403 (Trainer leave)</t>
-  </si>
-  <si>
     <t>FieldDTO[]</t>
-  </si>
-  <si>
-    <t>400 (Incomplete)</t>
-  </si>
-  <si>
-    <t>401 (Incomplete)</t>
   </si>
   <si>
     <t>Tout le monde</t>
@@ -595,12 +559,110 @@
   <si>
     <t>404 (Not found); 401(invalide)</t>
   </si>
+  <si>
+    <t>400 : identifiant invalide
+401 : non authentifié
+404 : utilisateur introuvable</t>
+  </si>
+  <si>
+    <t>400 : données invalides, email/username déjà pris
+401 : non authentifié
+403 : pas le propriétaire
+404 : utilisateur introuvable</t>
+  </si>
+  <si>
+    <t>401 : non authentifié ou rôle insuffisant</t>
+  </si>
+  <si>
+    <t>400 : status invalide
+401 : non authentifié
+403 : rôle insuffisant
+404 : utilisateur introuvable</t>
+  </si>
+  <si>
+    <t>400 : données invalides
+401 : non authentifié
+403 : rôle insuffisant
+404 : utilisateur introuvable</t>
+  </si>
+  <si>
+    <t>401 : non authentifié
+403 : rôle insuffisant</t>
+  </si>
+  <si>
+    <t>400 : données invalides,
+401 : non authentifié
+403 : rôle insuffisant
+404 : match introuvable</t>
+  </si>
+  <si>
+    <t>400 : match pas en status "started", scores invalides
+401 : non authentifié
+403 : rôle insuffisant
+404 : match introuvable</t>
+  </si>
+  <si>
+    <t>400 (Not started)</t>
+  </si>
+  <si>
+    <t>400 : identifiant invalide
+401 : non authentifié
+403 : rôle insuffisant
+404 : match introuvable</t>
+  </si>
+  <si>
+    <t>400 : champs manquants/invalides, nom déjà existant, sportType invalide
+401 : non authentifié
+403 : rôle insuffisant</t>
+  </si>
+  <si>
+    <t>400 : le trainer ne peut pas quitter l'équipe
+401 : non authentifié
+404 : équipe introuvable ou joueur pas dans l'équipe"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>403 (Trainer leave)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / 400 : utilisateur déjà dans l'équipe
+401 : non authentifié
+404 : équipe introuvable</t>
+    </r>
+  </si>
+  <si>
+    <t>400 : données invalides
+401 : non authentifié
+403 : pas le trainer de cette équipe
+404 : équipe introuvable</t>
+  </si>
+  <si>
+    <t>400 (Incomplete) 
+401 : non authentifié
+403 : rôle insuffisant</t>
+  </si>
+  <si>
+    <t>400 : identifiant invalide
+404 : terrain introuvable</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -725,6 +787,21 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -746,7 +823,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -840,11 +917,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB4C6E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB4C6E7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -875,9 +967,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -885,7 +974,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -911,7 +999,87 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1345,19 +1513,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6251F74D-515E-4B84-9C96-1B746F7F8599}">
   <sheetPr codeName="Feuil1"/>
   <dimension ref="A5:K30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.33203125" customWidth="1"/>
-    <col min="6" max="6" width="33.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" customWidth="1"/>
-    <col min="8" max="8" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="54.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="38.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.375" customWidth="1"/>
+    <col min="2" max="2" width="13.625" customWidth="1"/>
+    <col min="3" max="3" width="17.875" customWidth="1"/>
+    <col min="4" max="4" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.375" customWidth="1"/>
+    <col min="6" max="6" width="33.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.375" customWidth="1"/>
+    <col min="8" max="8" width="28.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="54.375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="38.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="33.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:11" ht="18">
@@ -1775,19 +1943,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E662E712-5C8B-461C-9C80-338D1AA5A420}">
   <sheetPr codeName="Feuil2"/>
   <dimension ref="A3:K66"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.21875" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" customWidth="1"/>
+    <col min="1" max="1" width="23.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.75" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="58.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="58.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:11" ht="18">
@@ -1825,22 +1993,22 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="21" t="s">
-        <v>133</v>
+    <row r="4" spans="1:11" ht="15">
+      <c r="A4" s="18" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="34" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="34" t="s">
         <v>35</v>
       </c>
       <c r="E5" s="11" t="s">
@@ -1859,7 +2027,7 @@
         <v>114</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="K5" t="s">
         <v>59</v>
@@ -1875,7 +2043,7 @@
       <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E6" s="11" t="s">
@@ -1885,7 +2053,7 @@
         <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H6" t="s">
         <v>60</v>
@@ -1894,7 +2062,7 @@
         <v>61</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="K6" t="s">
         <v>62</v>
@@ -1902,7 +2070,7 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -1910,8 +2078,8 @@
       <c r="C7" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="38" t="s">
-        <v>168</v>
+      <c r="D7" s="34" t="s">
+        <v>156</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>13</v>
@@ -1929,23 +2097,23 @@
         <v>63</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="K7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="40.200000000000003">
+    <row r="8" spans="1:11" ht="39.75">
       <c r="A8" t="s">
         <v>109</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="34" t="s">
         <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="34" t="s">
         <v>65</v>
       </c>
       <c r="E8" s="11" t="s">
@@ -1964,27 +2132,27 @@
         <v>116</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="K8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" ht="42.75">
       <c r="A9" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="34" t="s">
         <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="34" t="s">
         <v>67</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>13</v>
@@ -1999,156 +2167,159 @@
         <v>61</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="K9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="B10" s="24" t="s">
+    <row r="10" spans="1:11" s="40" customFormat="1" ht="71.25">
+      <c r="A10" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="24" t="s">
+      <c r="D10" s="41" t="s">
+        <v>140</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="I10" s="27" t="s">
+      <c r="I10" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="J10" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="K10" s="40" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:11" s="38" customFormat="1">
-      <c r="A11" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="B11" s="38" t="s">
+    <row r="11" spans="1:11" s="34" customFormat="1">
+      <c r="A11" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="38" t="s">
+      <c r="G11" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="I11" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="K11" s="38" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="12" t="s">
+      <c r="J11" s="36" t="s">
+        <v>165</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="57">
+      <c r="A12" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="37" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="G12" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="39" t="s">
         <v>74</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>61</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="K12" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="K12" s="39" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="38" customFormat="1">
-      <c r="A13" s="35" t="s">
+    <row r="13" spans="1:11" s="34" customFormat="1" ht="57">
+      <c r="A13" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="H13" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="J13" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="K13" s="43" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="26"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="12"/>
+    </row>
+    <row r="15" spans="1:11" s="21" customFormat="1" ht="15">
+      <c r="A15" s="27" t="s">
         <v>153</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>154</v>
-      </c>
-      <c r="E13" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="35" t="s">
-        <v>155</v>
-      </c>
-      <c r="H13" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" s="36" t="s">
-        <v>77</v>
-      </c>
-      <c r="J13" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="K13" s="40" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="12"/>
-    </row>
-    <row r="15" spans="1:11" s="24" customFormat="1">
-      <c r="A15" s="31" t="s">
-        <v>165</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2162,47 +2333,49 @@
       <c r="K15" s="12"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="32" t="s">
-        <v>169</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" s="32" t="s">
+      <c r="A16" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="C16" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="E16" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="32" t="s">
+      <c r="E16" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32" t="s">
+      <c r="H16" s="28"/>
+      <c r="I16" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="B17" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="J16" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" s="28" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="25.5">
+      <c r="A17" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="C17" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="44" t="s">
         <v>78</v>
       </c>
       <c r="E17" s="11" t="s">
@@ -2211,40 +2384,40 @@
       <c r="F17" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H17" s="37" t="s">
         <v>13</v>
       </c>
       <c r="I17" s="11" t="s">
         <v>81</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="K17" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K17" s="37" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="C18" s="12" t="s">
+    <row r="18" spans="1:11" ht="25.5">
+      <c r="A18" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="C18" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="44" t="s">
         <v>78</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="38" t="s">
         <v>41</v>
       </c>
       <c r="H18" s="12" t="s">
@@ -2253,43 +2426,43 @@
       <c r="I18" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J18" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="K18" s="12" t="s">
+      <c r="J18" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="K18" s="39" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="12" t="s">
+    <row r="19" spans="1:11" ht="57">
+      <c r="A19" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="44" t="s">
         <v>83</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="37" t="s">
         <v>84</v>
       </c>
       <c r="I19" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J19" s="13" t="s">
-        <v>123</v>
+      <c r="J19" s="55" t="s">
+        <v>169</v>
       </c>
       <c r="K19" s="12" t="s">
         <v>85</v>
@@ -2297,19 +2470,19 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="12" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="28" t="s">
         <v>86</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F20" s="11" t="s">
         <v>13</v>
@@ -2324,85 +2497,85 @@
         <v>81</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>124</v>
+        <v>171</v>
       </c>
       <c r="K20" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="12" t="s">
+    <row r="21" spans="1:11" ht="63.75">
+      <c r="A21" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="44" t="s">
         <v>90</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="H21" s="37" t="s">
         <v>91</v>
       </c>
       <c r="I21" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="J21" s="13" t="s">
+      <c r="J21" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="K21" s="37" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="51">
+      <c r="A22" s="39" t="s">
+        <v>132</v>
+      </c>
+      <c r="B22" s="45" t="s">
+        <v>138</v>
+      </c>
+      <c r="C22" s="45" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="K21" s="12" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="B22" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="C22" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>118</v>
-      </c>
       <c r="F22" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="12" t="s">
+      <c r="G22" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H22" s="39" t="s">
         <v>13</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="J22" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="K22" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="J22" s="49" t="s">
+        <v>172</v>
+      </c>
+      <c r="K22" s="37" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="22" customFormat="1">
-      <c r="A23" s="33" t="s">
-        <v>135</v>
+    <row r="23" spans="1:11" s="19" customFormat="1" ht="15">
+      <c r="A23" s="29" t="s">
+        <v>123</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -2416,30 +2589,30 @@
       <c r="K23" s="12"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="32"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="6" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="25" t="s">
-        <v>136</v>
+      <c r="D25" s="22" t="s">
+        <v>124</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>13</v>
@@ -2453,168 +2626,170 @@
       <c r="H25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I25" s="23" t="s">
+      <c r="I25" s="20" t="s">
         <v>95</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>125</v>
+        <v>13</v>
       </c>
       <c r="K25" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:11" ht="57">
+      <c r="A26" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="48" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="50" t="s">
         <v>94</v>
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="48" t="s">
         <v>98</v>
       </c>
       <c r="I26" s="16" t="s">
         <v>99</v>
       </c>
       <c r="J26" s="17" t="s">
-        <v>126</v>
+        <v>173</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B27" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="C27" s="2" t="s">
+    <row r="27" spans="1:11" ht="57">
+      <c r="A27" s="52" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="53" t="s">
+        <v>128</v>
+      </c>
+      <c r="C27" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="D27" s="53" t="s">
         <v>101</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="54" t="s">
         <v>13</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>99</v>
       </c>
       <c r="J27" s="15" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="28" spans="1:11" s="24" customFormat="1">
-      <c r="A28" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="C28" s="4" t="s">
+    <row r="28" spans="1:11" s="21" customFormat="1" ht="51">
+      <c r="A28" s="51" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="50" t="s">
         <v>101</v>
       </c>
       <c r="E28" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="I28" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="F28" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>128</v>
-      </c>
       <c r="J28" s="16" t="s">
-        <v>13</v>
+        <v>174</v>
       </c>
       <c r="K28" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="29" spans="1:11" s="24" customFormat="1">
-      <c r="A29" s="32" t="s">
-        <v>161</v>
-      </c>
-      <c r="B29" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="C29" s="32" t="s">
+    <row r="29" spans="1:11" s="21" customFormat="1" ht="51">
+      <c r="A29" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="B29" s="44" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="32" t="s">
-        <v>136</v>
-      </c>
-      <c r="E29" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="F29" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="32" t="s">
+      <c r="D29" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="E29" s="44" t="s">
+        <v>117</v>
+      </c>
+      <c r="F29" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="32" t="s">
+      <c r="H29" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="I29" s="32" t="s">
-        <v>137</v>
-      </c>
-      <c r="J29" s="32"/>
-      <c r="K29" s="32" t="s">
-        <v>138</v>
+      <c r="I29" s="44" t="s">
+        <v>125</v>
+      </c>
+      <c r="J29" s="56" t="s">
+        <v>176</v>
+      </c>
+      <c r="K29" s="28" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="32"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-    </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="33" t="s">
-        <v>158</v>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+    </row>
+    <row r="31" spans="1:11" ht="15">
+      <c r="A31" s="29" t="s">
+        <v>146</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -2627,17 +2802,17 @@
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
     </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="6" t="s">
+    <row r="32" spans="1:11" ht="42.75">
+      <c r="A32" s="52" t="s">
         <v>113</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="B32" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="54" t="s">
         <v>104</v>
       </c>
       <c r="E32" s="14" t="s">
@@ -2646,19 +2821,19 @@
       <c r="F32" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="54" t="s">
         <v>73</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="54" t="s">
         <v>105</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>106</v>
       </c>
       <c r="J32" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="K32" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="K32" s="57" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2678,15 +2853,17 @@
         <v>13</v>
       </c>
       <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
+      <c r="J33" s="16" t="s">
+        <v>13</v>
+      </c>
       <c r="K33" s="5"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="6" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
@@ -2701,148 +2878,148 @@
         <v>13</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>13</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="J34" s="15" t="s">
-        <v>130</v>
+        <v>118</v>
+      </c>
+      <c r="J34" s="58" t="s">
+        <v>13</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="B35" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="C35" s="19" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="28.5">
+      <c r="A35" s="61" t="s">
+        <v>151</v>
+      </c>
+      <c r="B35" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="C35" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="E35" s="12" t="s">
+      <c r="D35" s="60" t="s">
+        <v>150</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="F35" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="60" t="s">
+        <v>119</v>
+      </c>
+      <c r="H35" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="I35" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="F35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I35" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="J35" s="12">
-        <v>401</v>
-      </c>
-      <c r="K35" s="20" t="s">
-        <v>159</v>
+      <c r="J35" s="59" t="s">
+        <v>178</v>
+      </c>
+      <c r="K35" s="62" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="36" spans="1:11">
-      <c r="I36" s="39"/>
+      <c r="I36" s="35"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="I37" s="39"/>
+      <c r="I37" s="35"/>
     </row>
     <row r="38" spans="1:11">
-      <c r="I38" s="39"/>
+      <c r="I38" s="35"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="I39" s="39"/>
+      <c r="I39" s="35"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="I40" s="39"/>
+      <c r="I40" s="35"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="I41" s="39"/>
+      <c r="I41" s="35"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="I42" s="39"/>
+      <c r="I42" s="35"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="I43" s="39"/>
+      <c r="I43" s="35"/>
     </row>
     <row r="44" spans="1:11">
-      <c r="I44" s="39"/>
+      <c r="I44" s="35"/>
     </row>
     <row r="45" spans="1:11">
-      <c r="I45" s="39"/>
+      <c r="I45" s="35"/>
     </row>
     <row r="46" spans="1:11">
-      <c r="I46" s="39"/>
+      <c r="I46" s="35"/>
     </row>
     <row r="47" spans="1:11">
-      <c r="I47" s="39"/>
+      <c r="I47" s="35"/>
     </row>
     <row r="48" spans="1:11">
-      <c r="I48" s="39"/>
+      <c r="I48" s="35"/>
     </row>
     <row r="49" spans="9:9">
-      <c r="I49" s="39"/>
+      <c r="I49" s="35"/>
     </row>
     <row r="50" spans="9:9">
-      <c r="I50" s="39"/>
+      <c r="I50" s="35"/>
     </row>
     <row r="51" spans="9:9">
-      <c r="I51" s="39"/>
+      <c r="I51" s="35"/>
     </row>
     <row r="52" spans="9:9">
-      <c r="I52" s="39"/>
+      <c r="I52" s="35"/>
     </row>
     <row r="53" spans="9:9">
-      <c r="I53" s="39"/>
+      <c r="I53" s="35"/>
     </row>
     <row r="54" spans="9:9">
-      <c r="I54" s="39"/>
+      <c r="I54" s="35"/>
     </row>
     <row r="55" spans="9:9">
-      <c r="I55" s="39"/>
+      <c r="I55" s="35"/>
     </row>
     <row r="56" spans="9:9">
-      <c r="I56" s="39"/>
+      <c r="I56" s="35"/>
     </row>
     <row r="57" spans="9:9">
-      <c r="I57" s="39"/>
+      <c r="I57" s="35"/>
     </row>
     <row r="58" spans="9:9">
-      <c r="I58" s="39"/>
+      <c r="I58" s="35"/>
     </row>
     <row r="59" spans="9:9">
-      <c r="I59" s="39"/>
+      <c r="I59" s="35"/>
     </row>
     <row r="60" spans="9:9">
-      <c r="I60" s="39"/>
+      <c r="I60" s="35"/>
     </row>
     <row r="61" spans="9:9">
-      <c r="I61" s="39"/>
+      <c r="I61" s="35"/>
     </row>
     <row r="62" spans="9:9">
-      <c r="I62" s="39"/>
+      <c r="I62" s="35"/>
     </row>
     <row r="63" spans="9:9">
-      <c r="I63" s="39"/>
+      <c r="I63" s="35"/>
     </row>
     <row r="64" spans="9:9">
-      <c r="I64" s="39"/>
+      <c r="I64" s="35"/>
     </row>
     <row r="65" spans="9:9">
-      <c r="I65" s="39"/>
+      <c r="I65" s="35"/>
     </row>
     <row r="66" spans="9:9">
-      <c r="I66" s="39"/>
+      <c r="I66" s="35"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>